<commit_message>
Icon changes and new products
</commit_message>
<xml_diff>
--- a/data_from_insta/instagram_media_curatedkadha_20260822_043644.xlsx
+++ b/data_from_insta/instagram_media_curatedkadha_20260822_043644.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aucklandtransport-my.sharepoint.com/personal/nivin_johnson_at_govt_nz/Documents/Desktop/Exercise Files/Insta API/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aucklandtransport-my.sharepoint.com/personal/nivin_johnson_at_govt_nz/Documents/Desktop/Exercise Files/CuratedKadha/data_from_insta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_3D796E3C937E3045E901CCF0505ED87656C14522" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{471268EC-0C8D-4B0C-B64D-B3E46B04F744}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_3D796E3C937E3045E901CCF0505ED87656C14522" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1696814E-2A7E-4E37-8722-8F4963C0D284}"/>
   <bookViews>
-    <workbookView xWindow="13830" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14970" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="instagram_images" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5061" uniqueCount="3439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5182" uniqueCount="3516">
   <si>
     <t>record_id</t>
   </si>
@@ -11497,6 +11497,241 @@
   </si>
   <si>
     <t>https://scontent-akl1-1.cdninstagram.com/v/t51.75761-15/514905203_17847224832509801_6694969737507050620_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=110&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiRkVFRC5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=b3vAB601ucQQ7kNvwHVQfRS&amp;_nc_oc=AdolyRa228yJ-Lr8ueyXTy2YURVQ3vOzqL28nCWFE_f74ueIdIaLAOj86mTHyZtXNBc&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ANo9K5cEAAAA&amp;_nc_gid=K9l6TL5Odwv8FvgqXGXaxg&amp;_nc_tpa=Q5bMBQIXmhAkaBjAg7om158sBhfqqPEKEVHW8zlGpml8k_k7SCHdGxbSDxnS04sAC4kOtUbEBpEB6MA06w&amp;oh=00_AQEH8ZI1ofK-eIGlhjOilEcYv1KOF-XkuasgMnWeuSKkww&amp;oe=6A8F1331</t>
+  </si>
+  <si>
+    <t>17953571034219167_17909281449281956</t>
+  </si>
+  <si>
+    <t>17953571034219167</t>
+  </si>
+  <si>
+    <t>17909281449281956</t>
+  </si>
+  <si>
+    <t>17953571034219167_17909281449281956.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\17953571034219167_17909281449281956.jpg</t>
+  </si>
+  <si>
+    <t>L XL &amp; 2XL dress with pockets
+DM US</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYaKkFyx-6/</t>
+  </si>
+  <si>
+    <t>2026-08-23T11:44:25+0000</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/784222364_17903783265509801_3344793913947769257_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=106&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=xg9cjwhfUHwQ7kNvwFYKfTW&amp;_nc_oc=AdpQ5WcGNxlI8gFIkF7uWVCrUfzlxb0KL9-QUbI7tRaUtbRVPWW6sUUsz01-CYAbWNw&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=ZtsoNF3ZhjTllvlpxaBThg&amp;_nc_tpa=Q5bMBQK383xam3vPnIMNU49ynVBirCdhxTio5MmkOCPjlHKr9Ijxw1JJmNdgbwbVUg7agEuVlXgAi8iWUQ&amp;oh=00_AQJ6JtF54ObGmdGfeh7t6MaD-IyerbyaumBGbIxD0hzKDg&amp;oe=6A9A7BE5</t>
+  </si>
+  <si>
+    <t>17953571034219167_18089176112555363</t>
+  </si>
+  <si>
+    <t>18089176112555363</t>
+  </si>
+  <si>
+    <t>17953571034219167_18089176112555363.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\17953571034219167_18089176112555363.jpg</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYaKo6S3nc/</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/781630256_17903783277509801_3028076470035516603_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=110&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=IW40hBKqGVoQ7kNvwGh-H26&amp;_nc_oc=AdpU3jREtVYKz92bUCQfZHvVXNtTgb1IYLSl2iCa5l8hTEe7B_muMVyjPiynBx0BewE&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=ZtsoNF3ZhjTllvlpxaBThg&amp;_nc_tpa=Q5bMBQKJuNYjN1vE6vuBAXjy_VmvxDlv7k7kj7zDAgsBbKIBnBIUfJr6Waugzd8dVhTkBCc4p9wvY3F3cg&amp;oh=00_AQJ44XNFKDSI74hVEiu0w3fW3VwYXPzU99MvM_xOv9Y4Mg&amp;oe=6A9A9445</t>
+  </si>
+  <si>
+    <t>17953571034219167_18048633269593817</t>
+  </si>
+  <si>
+    <t>18048633269593817</t>
+  </si>
+  <si>
+    <t>17953571034219167_18048633269593817.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\17953571034219167_18048633269593817.jpg</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYaKtuy2pQ/</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/784250688_17903783286509801_6469293784245415839_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=106&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=ThQAbMzaZe0Q7kNvwEbhsYz&amp;_nc_oc=AdrBcWIg6VLM1sTquulfvYMSQMMNxAr7wZkr8MGxsCvMTOVzepxzIPVEMwQy1zwmRfM&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=ZtsoNF3ZhjTllvlpxaBThg&amp;_nc_tpa=Q5bMBQJ4f4lssY1nRZ4a7XrfBXnF015sWnw7FzT_FJ95avE5EZ6D2lbojJrSAWNtXFfQoKEe9_0UOFlW6g&amp;oh=00_AQK3RCzsGBugDJY8denAKa8PKgnTkUbuNl5oVIwWnYZvwA&amp;oe=6A9A8A42</t>
+  </si>
+  <si>
+    <t>18177675028437927_17903511075327398</t>
+  </si>
+  <si>
+    <t>18177675028437927</t>
+  </si>
+  <si>
+    <t>17903511075327398</t>
+  </si>
+  <si>
+    <t>18177675028437927_17903511075327398.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\18177675028437927_17903511075327398.jpg</t>
+  </si>
+  <si>
+    <t>❌SOLD❌
+Large SOLD &amp; XL SOLD size dress with pockets
+DM US</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYaC_ySBnD/</t>
+  </si>
+  <si>
+    <t>2026-08-23T11:43:34+0000</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/781459579_17903782791509801_2817349832938121073_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=107&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=bc3qi1u9GHIQ7kNvwHAxQLL&amp;_nc_oc=AdrC1aoXAAwsrssAxSe0evR14wtaff6nNcjw2LuPOJHfPq3st0XhvE_yay-5zhpymMs&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=BoRqeLCH3DfYf5mYJXrEdw&amp;_nc_tpa=Q5bMBQLLmiL1w2vKBhd2JFj8J23tzTqCTS6iU_Lptq2ADWg_biFg97LXqKJAVY8g3QGzbat8iiQS0p9Wdw&amp;oh=00_AQIalkwBzVbSve8H54ia2QmdN9Lndxu1fOi9blkB03EMjw&amp;oe=6A9AA8B7</t>
+  </si>
+  <si>
+    <t>18177675028437927_17974121243925001</t>
+  </si>
+  <si>
+    <t>17974121243925001</t>
+  </si>
+  <si>
+    <t>18177675028437927_17974121243925001.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\18177675028437927_17974121243925001.jpg</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYaDMUyyL1/</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/782599020_17903782806509801_3119522399240640470_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=107&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=OE0K7yt5P9kQ7kNvwEcJV94&amp;_nc_oc=AdpO2EPZ7u48kF7FQTRBFstmP_LT6NFgeHgTxTcHtGC-qdwbmd0mKSiSEgowIHSflZo&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=BoRqeLCH3DfYf5mYJXrEdw&amp;_nc_tpa=Q5bMBQLjWJ5797WcbzPR8wKo_5NDMVfhidy70yio1ZyjwOgd70BASYhNLSMbNFt_HfJQyys01RfW_CMIOg&amp;oh=00_AQIj-gTzyBXHAvf-JKIkkAvxb73wK90TSDls3QPqeziFiA&amp;oe=6A9A9ED6</t>
+  </si>
+  <si>
+    <t>18177675028437927_18450689305187068</t>
+  </si>
+  <si>
+    <t>18450689305187068</t>
+  </si>
+  <si>
+    <t>18177675028437927_18450689305187068.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\18177675028437927_18450689305187068.jpg</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYaDSMSy7T/</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/782252213_17903782824509801_5072783778858894737_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=107&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=LgEPTjf_dJkQ7kNvwGts6SD&amp;_nc_oc=AdpSYXnLgTdRIpKvbKWP0aqdz_lL4BVNx074Y2-11ws8xQX9FNDTyQIAGMusIOGltoA&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=BoRqeLCH3DfYf5mYJXrEdw&amp;_nc_tpa=Q5bMBQLgeFwwWBZU4RIAigrCAbD7QEv5qvTw8_KECOxegcRF3TagLOqGLeAUQ2IFOQo2b9_NKSWxfj_wlQ&amp;oh=00_AQJGZ7If8DnfQoF1GnvrAKAAj2q1hkvWrYgtlLNrt3WwpA&amp;oe=6A9A9E4B</t>
+  </si>
+  <si>
+    <t>18177675028437927_17926966455164099</t>
+  </si>
+  <si>
+    <t>17926966455164099</t>
+  </si>
+  <si>
+    <t>18177675028437927_17926966455164099.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\18177675028437927_17926966455164099.jpg</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYaDWWyvtR/</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/783205220_17903782833509801_541611849486016587_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=108&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=QcYlJyzYwaEQ7kNvwHHEP6T&amp;_nc_oc=AdoANqXzYhHUgW8xBwxjb4RK1x0ztF1BTgzTUqYgYPU30280tEWuSliB8GrfKjTcXFU&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=BoRqeLCH3DfYf5mYJXrEdw&amp;_nc_tpa=Q5bMBQK_AEwqTG0ZTWKrc8H1-3VXRDKed409jrAYFG59BA5UnHa2Cybj0vJoMc2ZqiNtxjvssl9upIaSYA&amp;oh=00_AQL2VaLni1dtLvCagQRwXKRDH-8ZFXy8FRbP6N-J-TLwwQ&amp;oe=6A9A8D6A</t>
+  </si>
+  <si>
+    <t>17897054475378053_18389246230166275</t>
+  </si>
+  <si>
+    <t>17897054475378053</t>
+  </si>
+  <si>
+    <t>18389246230166275</t>
+  </si>
+  <si>
+    <t>17897054475378053_18389246230166275.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\17897054475378053_18389246230166275.jpg</t>
+  </si>
+  <si>
+    <t>Large size dress
+DM US</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYZ9r8SjU4/</t>
+  </si>
+  <si>
+    <t>2026-08-23T11:42:36+0000</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/784426226_17903782572509801_5464334519122490000_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=107&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=Js566aFzQdkQ7kNvwGY8fmt&amp;_nc_oc=AdoTFjKEUdsHpSQS1ERFSlqywc-tE5MVSSngCzIU7l4upo-l2xZ3-ArUXFMdLouwhnc&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=iB5DoPTtM2zFuGnLT7GfqA&amp;_nc_tpa=Q5bMBQJ2t6oVbkK6xKh01tcvhfmluLV1YQTpoD94RK3WmclAiPpOiCt2B9Xivkk8zXQOwUy2kvjPn4Mqtg&amp;oh=00_AQIHWKDYnyWHBYmdWOQkhyZL5rROXKXDi5Lpj-egRPcQdA&amp;oe=6A9A90A3</t>
+  </si>
+  <si>
+    <t>17897054475378053_18622428223036299</t>
+  </si>
+  <si>
+    <t>18622428223036299</t>
+  </si>
+  <si>
+    <t>17897054475378053_18622428223036299.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\17897054475378053_18622428223036299.jpg</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYZ91hywzK/</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/782252216_17903782602509801_5863334611908893379_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=102&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=xCMG_q8RursQ7kNvwHlQJqC&amp;_nc_oc=AdrKg5uijXIh1TM3_x_ZLS6DYHhp_cxgP8RZ1IEcHr1e04gaBbDJj3b22EecpKCxDwc&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=iB5DoPTtM2zFuGnLT7GfqA&amp;_nc_tpa=Q5bMBQKs6nKcWNxWvfMuFe23eV60tLQWp1yEqo7-3H1hK-UwBVtpgn6Q-JpukQfhxG6s8zleUWmbAp-lTg&amp;oh=00_AQK2E18qb9x8jhNWbyANYots6t87g7NA9lBuAP9yFlVahw&amp;oe=6A9A8748</t>
+  </si>
+  <si>
+    <t>18213597022342281_17960241915191788</t>
+  </si>
+  <si>
+    <t>18213597022342281</t>
+  </si>
+  <si>
+    <t>17960241915191788</t>
+  </si>
+  <si>
+    <t>18213597022342281_17960241915191788.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\18213597022342281_17960241915191788.jpg</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYZ2F_SuE_/</t>
+  </si>
+  <si>
+    <t>2026-08-23T11:41:43+0000</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/783707129_17903782398509801_6830695110993567785_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=106&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=vjZttM4VinsQ7kNvwFp9052&amp;_nc_oc=Ado2vWTw-T2wzJ1V6azCeIEO4VlP3H8W9fche9fsLVeh8OiwfqFSXKZfwlkWwh8pqmo&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=rFgkwfSTsIfuWuZDmHlqgw&amp;_nc_tpa=Q5bMBQLxSgk-bpqrS3mFDaTY7Pv_96nsFDCRn2K02CtdbFow-nDKdhI_1o3HvsuvatkNWYoT52BzL9kCEw&amp;oh=00_AQIhwUhn54d7vAhVCLIeaHpxwCQZ0TW8dpf57DtVVcBBgA&amp;oe=6A9A84DD</t>
+  </si>
+  <si>
+    <t>18213597022342281_17987031432047025</t>
+  </si>
+  <si>
+    <t>17987031432047025</t>
+  </si>
+  <si>
+    <t>18213597022342281_17987031432047025.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\NivinJoh1\OneDrive - Auckland Transport\Desktop\Exercise Files\Insta API\pictures\18213597022342281_17987031432047025.jpg</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DcYZ2PvySjk/</t>
+  </si>
+  <si>
+    <t>https://scontent-akl1-1.cdninstagram.com/v/t51.82787-15/782455825_17903782413509801_5797442859557385181_n.jpg?stp=dst-jpg_e35_tt6&amp;_nc_cat=101&amp;ccb=7-5&amp;_nc_sid=18de74&amp;efg=eyJlZmdfdGFnIjoiQ0FST1VTRUxfSVRFTS5iZXN0X2ltYWdlX3VybGdlbi5DMyJ9&amp;_nc_ohc=4DMSEzq_jmYQ7kNvwEPu3bi&amp;_nc_oc=Adq6Z5-EXZ5zCetUK3MHCwQDRBV2pPe-WoaCPO6jma2BQdB1XxAIoo8rFQgoGW9aGNc&amp;_nc_zt=23&amp;_nc_ht=scontent-akl1-1.cdninstagram.com&amp;edm=ABbrh9MEAAAA&amp;_nc_gid=rFgkwfSTsIfuWuZDmHlqgw&amp;_nc_tpa=Q5bMBQJfS91WhagP0NiRreRv56w5LS0uEppfgXPemukGTLcbjPmIUCmJljzy3qdkz61VFQep-AYB6x2QVA&amp;oh=00_AQJt_TAdvagcCOQ3_1VszbMwm3CN2wOjj5SBG6-0O6PvCg&amp;oe=6A9A9D4C</t>
   </si>
 </sst>
 </file>
@@ -11836,7 +12071,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L460"/>
+  <dimension ref="A1:L471"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36.81640625" customWidth="1"/>
@@ -27952,6 +28187,391 @@
         <v>22</v>
       </c>
     </row>
+    <row r="461" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A461" t="s">
+        <v>3439</v>
+      </c>
+      <c r="B461" t="s">
+        <v>3440</v>
+      </c>
+      <c r="C461" t="s">
+        <v>3441</v>
+      </c>
+      <c r="D461" t="s">
+        <v>15</v>
+      </c>
+      <c r="E461" t="s">
+        <v>3442</v>
+      </c>
+      <c r="F461" t="s">
+        <v>3443</v>
+      </c>
+      <c r="G461" t="s">
+        <v>3444</v>
+      </c>
+      <c r="H461" t="s">
+        <v>3445</v>
+      </c>
+      <c r="I461" t="s">
+        <v>3446</v>
+      </c>
+      <c r="J461" t="s">
+        <v>3447</v>
+      </c>
+      <c r="K461" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="462" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A462" t="s">
+        <v>3448</v>
+      </c>
+      <c r="B462" t="s">
+        <v>3440</v>
+      </c>
+      <c r="C462" t="s">
+        <v>3449</v>
+      </c>
+      <c r="D462" t="s">
+        <v>15</v>
+      </c>
+      <c r="E462" t="s">
+        <v>3450</v>
+      </c>
+      <c r="F462" t="s">
+        <v>3451</v>
+      </c>
+      <c r="G462" t="s">
+        <v>3444</v>
+      </c>
+      <c r="H462" t="s">
+        <v>3452</v>
+      </c>
+      <c r="I462" t="s">
+        <v>3446</v>
+      </c>
+      <c r="J462" t="s">
+        <v>3453</v>
+      </c>
+      <c r="K462" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="463" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A463" t="s">
+        <v>3454</v>
+      </c>
+      <c r="B463" t="s">
+        <v>3440</v>
+      </c>
+      <c r="C463" t="s">
+        <v>3455</v>
+      </c>
+      <c r="D463" t="s">
+        <v>15</v>
+      </c>
+      <c r="E463" t="s">
+        <v>3456</v>
+      </c>
+      <c r="F463" t="s">
+        <v>3457</v>
+      </c>
+      <c r="G463" t="s">
+        <v>3444</v>
+      </c>
+      <c r="H463" t="s">
+        <v>3458</v>
+      </c>
+      <c r="I463" t="s">
+        <v>3446</v>
+      </c>
+      <c r="J463" t="s">
+        <v>3459</v>
+      </c>
+      <c r="K463" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="464" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A464" t="s">
+        <v>3460</v>
+      </c>
+      <c r="B464" t="s">
+        <v>3461</v>
+      </c>
+      <c r="C464" t="s">
+        <v>3462</v>
+      </c>
+      <c r="D464" t="s">
+        <v>15</v>
+      </c>
+      <c r="E464" t="s">
+        <v>3463</v>
+      </c>
+      <c r="F464" t="s">
+        <v>3464</v>
+      </c>
+      <c r="G464" t="s">
+        <v>3465</v>
+      </c>
+      <c r="H464" t="s">
+        <v>3466</v>
+      </c>
+      <c r="I464" t="s">
+        <v>3467</v>
+      </c>
+      <c r="J464" t="s">
+        <v>3468</v>
+      </c>
+      <c r="K464" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="465" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A465" t="s">
+        <v>3469</v>
+      </c>
+      <c r="B465" t="s">
+        <v>3461</v>
+      </c>
+      <c r="C465" t="s">
+        <v>3470</v>
+      </c>
+      <c r="D465" t="s">
+        <v>15</v>
+      </c>
+      <c r="E465" t="s">
+        <v>3471</v>
+      </c>
+      <c r="F465" t="s">
+        <v>3472</v>
+      </c>
+      <c r="G465" t="s">
+        <v>3465</v>
+      </c>
+      <c r="H465" t="s">
+        <v>3473</v>
+      </c>
+      <c r="I465" t="s">
+        <v>3467</v>
+      </c>
+      <c r="J465" t="s">
+        <v>3474</v>
+      </c>
+      <c r="K465" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="466" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A466" t="s">
+        <v>3475</v>
+      </c>
+      <c r="B466" t="s">
+        <v>3461</v>
+      </c>
+      <c r="C466" t="s">
+        <v>3476</v>
+      </c>
+      <c r="D466" t="s">
+        <v>15</v>
+      </c>
+      <c r="E466" t="s">
+        <v>3477</v>
+      </c>
+      <c r="F466" t="s">
+        <v>3478</v>
+      </c>
+      <c r="G466" t="s">
+        <v>3465</v>
+      </c>
+      <c r="H466" t="s">
+        <v>3479</v>
+      </c>
+      <c r="I466" t="s">
+        <v>3467</v>
+      </c>
+      <c r="J466" t="s">
+        <v>3480</v>
+      </c>
+      <c r="K466" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="467" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A467" t="s">
+        <v>3481</v>
+      </c>
+      <c r="B467" t="s">
+        <v>3461</v>
+      </c>
+      <c r="C467" t="s">
+        <v>3482</v>
+      </c>
+      <c r="D467" t="s">
+        <v>15</v>
+      </c>
+      <c r="E467" t="s">
+        <v>3483</v>
+      </c>
+      <c r="F467" t="s">
+        <v>3484</v>
+      </c>
+      <c r="G467" t="s">
+        <v>3465</v>
+      </c>
+      <c r="H467" t="s">
+        <v>3485</v>
+      </c>
+      <c r="I467" t="s">
+        <v>3467</v>
+      </c>
+      <c r="J467" t="s">
+        <v>3486</v>
+      </c>
+      <c r="K467" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="468" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A468" t="s">
+        <v>3487</v>
+      </c>
+      <c r="B468" t="s">
+        <v>3488</v>
+      </c>
+      <c r="C468" t="s">
+        <v>3489</v>
+      </c>
+      <c r="D468" t="s">
+        <v>15</v>
+      </c>
+      <c r="E468" t="s">
+        <v>3490</v>
+      </c>
+      <c r="F468" t="s">
+        <v>3491</v>
+      </c>
+      <c r="G468" t="s">
+        <v>3492</v>
+      </c>
+      <c r="H468" t="s">
+        <v>3493</v>
+      </c>
+      <c r="I468" t="s">
+        <v>3494</v>
+      </c>
+      <c r="J468" t="s">
+        <v>3495</v>
+      </c>
+      <c r="K468" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="469" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A469" t="s">
+        <v>3496</v>
+      </c>
+      <c r="B469" t="s">
+        <v>3488</v>
+      </c>
+      <c r="C469" t="s">
+        <v>3497</v>
+      </c>
+      <c r="D469" t="s">
+        <v>15</v>
+      </c>
+      <c r="E469" t="s">
+        <v>3498</v>
+      </c>
+      <c r="F469" t="s">
+        <v>3499</v>
+      </c>
+      <c r="G469" t="s">
+        <v>3492</v>
+      </c>
+      <c r="H469" t="s">
+        <v>3500</v>
+      </c>
+      <c r="I469" t="s">
+        <v>3494</v>
+      </c>
+      <c r="J469" t="s">
+        <v>3501</v>
+      </c>
+      <c r="K469" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="470" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A470" t="s">
+        <v>3502</v>
+      </c>
+      <c r="B470" t="s">
+        <v>3503</v>
+      </c>
+      <c r="C470" t="s">
+        <v>3504</v>
+      </c>
+      <c r="D470" t="s">
+        <v>15</v>
+      </c>
+      <c r="E470" t="s">
+        <v>3505</v>
+      </c>
+      <c r="F470" t="s">
+        <v>3506</v>
+      </c>
+      <c r="G470" t="s">
+        <v>3492</v>
+      </c>
+      <c r="H470" t="s">
+        <v>3507</v>
+      </c>
+      <c r="I470" t="s">
+        <v>3508</v>
+      </c>
+      <c r="J470" t="s">
+        <v>3509</v>
+      </c>
+      <c r="K470" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="471" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A471" t="s">
+        <v>3510</v>
+      </c>
+      <c r="B471" t="s">
+        <v>3503</v>
+      </c>
+      <c r="C471" t="s">
+        <v>3511</v>
+      </c>
+      <c r="D471" t="s">
+        <v>15</v>
+      </c>
+      <c r="E471" t="s">
+        <v>3512</v>
+      </c>
+      <c r="F471" t="s">
+        <v>3513</v>
+      </c>
+      <c r="G471" t="s">
+        <v>3492</v>
+      </c>
+      <c r="H471" t="s">
+        <v>3514</v>
+      </c>
+      <c r="I471" t="s">
+        <v>3508</v>
+      </c>
+      <c r="J471" t="s">
+        <v>3515</v>
+      </c>
+      <c r="K471" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>